<commit_message>
not working yet... but soon
</commit_message>
<xml_diff>
--- a/public/catalog.xlsx
+++ b/public/catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/astrid/GitHub/personal-portfolio/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F41C65-1687-EE47-85C3-3F371E3C85E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6DB741B-2535-B04D-BBA0-0651F103E144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="18480" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="78">
   <si>
     <t>file</t>
   </si>
@@ -236,6 +236,24 @@
   </si>
   <si>
     <t>[more]</t>
+  </si>
+  <si>
+    <t>canvas-a.jpg</t>
+  </si>
+  <si>
+    <t>canvas-b.jpg</t>
+  </si>
+  <si>
+    <t>59 × 60 in</t>
+  </si>
+  <si>
+    <t>60 × 60 in</t>
+  </si>
+  <si>
+    <t>layout</t>
+  </si>
+  <si>
+    <t>offset</t>
   </si>
 </sst>
 </file>
@@ -618,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
@@ -627,9 +645,10 @@
     <col min="5" max="5" width="28.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="38.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -654,8 +673,11 @@
       <c r="H1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -678,7 +700,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -698,7 +720,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -721,7 +743,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -741,7 +763,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>48</v>
       </c>
@@ -764,7 +786,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -787,7 +809,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>50</v>
       </c>
@@ -810,7 +832,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>51</v>
       </c>
@@ -830,7 +852,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>52</v>
       </c>
@@ -853,7 +875,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -876,7 +898,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -899,7 +921,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -922,7 +944,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>56</v>
       </c>
@@ -945,7 +967,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -968,7 +990,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>58</v>
       </c>
@@ -991,7 +1013,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -1014,7 +1036,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -1037,7 +1059,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>61</v>
       </c>
@@ -1060,7 +1082,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -1081,6 +1103,58 @@
       </c>
       <c r="H20" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21">
+        <v>2026</v>
+      </c>
+      <c r="D21">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" t="s">
+        <v>74</v>
+      </c>
+      <c r="H21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22">
+        <v>2026</v>
+      </c>
+      <c r="D22">
+        <v>7</v>
+      </c>
+      <c r="E22" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" t="s">
+        <v>75</v>
+      </c>
+      <c r="H22" t="s">
+        <v>69</v>
+      </c>
+      <c r="I22" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>